<commit_message>
Requirements: FR-90 reworked to manager + two group-level switches
Owner ruling (rev.4 item 5) replaces per-person writer marks:
- Every group has ONE manager (private: creator; organized: admin-assigned,
  must be a member). Manager always sees and writes, and is the only one
  who can flip the two switches.
- Visibility switch (all members / authority roles only): membership alone
  no longer grants chat access — a student is a department member yet does
  not see the department chat; their course chat (all-members) they do.
- Write switch (manager only / members too), default manager-only;
  organized initial values set by the admin, private chosen at creation.
- Seeing and writing are independent layers (academic sees the department
  chat read-only behind the lock bar).

Excel snapshots regenerated with Manager / Visibility / Members-can-write
columns.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/GroupConnect_Site_2026-07-19.xlsx
+++ b/docs/GroupConnect_Site_2026-07-19.xlsx
@@ -1504,15 +1504,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1543,7 +1544,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Yazar(lar)</t>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Üyeler Yazar mı</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1579,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Vedat Coşkun, Kemal Öztürk</t>
+          <t>Vedat Coşkun</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
         </is>
       </c>
     </row>
@@ -1606,6 +1617,11 @@
           <t>Vedat Coşkun</t>
         </is>
       </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1635,7 +1651,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>— (manager yok)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1688,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>— (manager yok)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
         </is>
       </c>
     </row>
@@ -1700,6 +1726,11 @@
           <t>Kerem Yalçın</t>
         </is>
       </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1730,6 +1761,11 @@
           <t>Tolga Erdem</t>
         </is>
       </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1759,7 +1795,12 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>— (manager yok)</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
         </is>
       </c>
     </row>
@@ -1792,6 +1833,11 @@
           <t>Pınar Çelik</t>
         </is>
       </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1822,6 +1868,11 @@
           <t>Gizem Polat</t>
         </is>
       </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1852,6 +1903,11 @@
           <t>Cem Yıldırım</t>
         </is>
       </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1882,6 +1938,11 @@
           <t>Ebru Kaplan</t>
         </is>
       </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1911,7 +1972,12 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>— (manager yok)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
         </is>
       </c>
     </row>
@@ -1943,7 +2009,12 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>— (manager yok)</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
         </is>
       </c>
     </row>
@@ -1976,6 +2047,11 @@
           <t>Derya Aksakal</t>
         </is>
       </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2005,7 +2081,12 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>— (manager yok)</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
         </is>
       </c>
     </row>
@@ -2036,6 +2117,11 @@
       <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Volkan Tunç</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Hayır</t>
         </is>
       </c>
     </row>

</xml_diff>